<commit_message>
Update: Threat Alert Report - 2026-05-18 13:48
</commit_message>
<xml_diff>
--- a/excel_routes/route_AJF_CAI_threats.xlsx
+++ b/excel_routes/route_AJF_CAI_threats.xlsx
@@ -33,7 +33,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -44,6 +44,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="003498DB"/>
         <bgColor rgb="003498DB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF3CD"/>
+        <bgColor rgb="00FFF3CD"/>
       </patternFill>
     </fill>
     <fill>
@@ -71,7 +77,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -80,6 +86,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -540,10 +549,10 @@
         <v>950</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>1098</v>
+        <v>1189</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>-148</v>
+        <v>-239</v>
       </c>
       <c r="G2" s="2" t="n">
         <v>30</v>
@@ -556,7 +565,7 @@
       </c>
       <c r="J2" s="3" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>MED</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -599,7 +608,7 @@
       <c r="I3" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="J3" s="3" t="inlineStr">
+      <c r="J3" s="4" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
@@ -644,7 +653,7 @@
       <c r="I4" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="J4" s="3" t="inlineStr">
+      <c r="J4" s="4" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
@@ -689,7 +698,7 @@
       <c r="I5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="J5" s="3" t="inlineStr">
+      <c r="J5" s="4" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
@@ -734,7 +743,7 @@
       <c r="I6" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="J6" s="3" t="inlineStr">
+      <c r="J6" s="4" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
@@ -779,7 +788,7 @@
       <c r="I7" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="J7" s="3" t="inlineStr">
+      <c r="J7" s="4" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
@@ -824,7 +833,7 @@
       <c r="I8" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="J8" s="3" t="inlineStr">
+      <c r="J8" s="4" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
@@ -869,7 +878,7 @@
       <c r="I9" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="J9" s="3" t="inlineStr">
+      <c r="J9" s="4" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
@@ -914,7 +923,7 @@
       <c r="I10" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="J10" s="3" t="inlineStr">
+      <c r="J10" s="4" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
@@ -959,7 +968,7 @@
       <c r="I11" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="J11" s="3" t="inlineStr">
+      <c r="J11" s="4" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
@@ -1004,7 +1013,7 @@
       <c r="I12" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="J12" s="3" t="inlineStr">
+      <c r="J12" s="4" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
@@ -1049,7 +1058,7 @@
       <c r="I13" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="J13" s="3" t="inlineStr">
+      <c r="J13" s="4" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
@@ -1094,7 +1103,7 @@
       <c r="I14" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="J14" s="3" t="inlineStr">
+      <c r="J14" s="4" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
@@ -1139,7 +1148,7 @@
       <c r="I15" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="J15" s="3" t="inlineStr">
+      <c r="J15" s="4" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>

</xml_diff>